<commit_message>
Update imports data excel
</commit_message>
<xml_diff>
--- a/sqms_apps/static/format-upload/template-import-sellings-hos.xlsx
+++ b/sqms_apps/static/format-upload/template-import-sellings-hos.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meinardus.bria\Desktop\SQMS - Python imports\format-downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meinardus.bria\django_project\alpha\sqms_apps\static\format-upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634DF7F6-BC02-4CD8-9329-4A38BD85CC64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F05B8C7-4280-4135-BCA6-4CCC493A66D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{164D2D34-7551-47B0-9F6A-8815E64D8F5F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{164D2D34-7551-47B0-9F6A-8815E64D8F5F}"/>
   </bookViews>
   <sheets>
     <sheet name="import-hos" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'import-hos'!$A$1:$S$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'import-hos'!$A$1:$R$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
     <author>Meinardus Bria</author>
   </authors>
   <commentList>
-    <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{D6F9940C-3F8B-4EE9-A75F-2D54A974B936}">
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{D6F9940C-3F8B-4EE9-A75F-2D54A974B936}">
       <text>
         <r>
           <rPr>
@@ -68,7 +68,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0" xr:uid="{88FCD418-98A7-4B20-BA7A-64759DC865B9}">
+    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{88FCD418-98A7-4B20-BA7A-64759DC865B9}">
       <text>
         <r>
           <rPr>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>shift</t>
   </si>
@@ -138,9 +138,6 @@
     <t>berat_kosong</t>
   </si>
   <si>
-    <t>stockpile</t>
-  </si>
-  <si>
     <t>dome</t>
   </si>
   <si>
@@ -169,9 +166,6 @@
   </si>
   <si>
     <t>L9_02</t>
-  </si>
-  <si>
-    <t>LS_09</t>
   </si>
   <si>
     <t>FPP_HY</t>
@@ -334,7 +328,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -346,7 +340,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -354,28 +347,27 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -397,10 +389,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -700,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{675D438A-BC23-488B-AFE3-E8314FA5CCB8}">
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.7109375" style="1" customWidth="1"/>
@@ -714,300 +702,285 @@
     <col min="9" max="9" width="18.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.7109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="8.140625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.42578125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" style="3" customWidth="1"/>
-    <col min="17" max="17" width="10.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.85546875" style="1"/>
+    <col min="12" max="12" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.42578125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.42578125" style="3" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="O1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
         <v>18</v>
       </c>
+      <c r="B2" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="9">
+        <v>54580</v>
+      </c>
+      <c r="E2" s="9">
+        <v>20280</v>
+      </c>
+      <c r="F2" s="9">
+        <v>34300</v>
+      </c>
+      <c r="G2" s="12">
+        <v>45658.246203703704</v>
+      </c>
+      <c r="H2" s="12">
+        <v>45658.253912037035</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="13">
+        <v>45658</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q2" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="R2" s="17" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:19" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="11">
-        <v>54580</v>
-      </c>
-      <c r="E2" s="11">
-        <v>20280</v>
-      </c>
-      <c r="F2" s="11">
-        <v>34300</v>
-      </c>
-      <c r="G2" s="14">
-        <v>45658.246203703704</v>
-      </c>
-      <c r="H2" s="14">
-        <v>45658.253912037035</v>
-      </c>
-      <c r="I2" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="15">
-        <v>45658</v>
-      </c>
-      <c r="K2" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="P2" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q2" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="R2" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="S2" s="19" t="s">
-        <v>21</v>
-      </c>
+    <row r="3" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="9"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="17"/>
     </row>
-    <row r="3" spans="1:19" s="5" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="11"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="18"/>
-      <c r="S3" s="19"/>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="9"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="17"/>
     </row>
-    <row r="4" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="11"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="18"/>
-      <c r="S4" s="19"/>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="17"/>
     </row>
-    <row r="5" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="17"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="19"/>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="9"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="11"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="17"/>
     </row>
-    <row r="6" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="19"/>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A7" s="9"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="17"/>
     </row>
-    <row r="7" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="11"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="19"/>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A8" s="9"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="17"/>
     </row>
-    <row r="8" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="17"/>
-      <c r="Q8" s="13"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="19"/>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="9"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="17"/>
     </row>
-    <row r="9" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="17"/>
-      <c r="Q9" s="13"/>
-      <c r="R9" s="18"/>
-      <c r="S9" s="19"/>
-    </row>
-    <row r="10" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="16"/>
-      <c r="P10" s="17"/>
-      <c r="Q10" s="13"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="19"/>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" s="9"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>